<commit_message>
Add German guide localization
Generate static English and German online guides from shared templates and paired catalogs. Add localized worksheets and quick guides while retaining a single English BIP39 word list and an English-only offline edition.
</commit_message>
<xml_diff>
--- a/additional_ressources/BitsToWords.xlsx
+++ b/additional_ressources/BitsToWords.xlsx
@@ -49,7 +49,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -77,11 +77,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -167,7 +162,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -220,28 +215,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3161,12 +3152,12 @@
       <c r="AR18" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="AS18" s="18" t="s">
+      <c r="AS18" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="AT18" s="18"/>
-      <c r="AU18" s="18"/>
-      <c r="AV18" s="18"/>
+      <c r="AT18" s="13"/>
+      <c r="AU18" s="13"/>
+      <c r="AV18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="16"/>

</xml_diff>